<commit_message>
Update Comet subtype profile reporting
</commit_message>
<xml_diff>
--- a/Reference_seqs/HCV_GT_Ref_vs_Comet_GT_Consensus_Differences_NS5A_NTD.xlsx
+++ b/Reference_seqs/HCV_GT_Ref_vs_Comet_GT_Consensus_Differences_NS5A_NTD.xlsx
@@ -1590,7 +1590,7 @@
       <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>L</t>
         </is>
       </c>
       <c r="I28" t="inlineStr"/>
@@ -1598,7 +1598,11 @@
       <c r="K28" t="inlineStr"/>
       <c r="L28" t="inlineStr"/>
       <c r="M28" t="inlineStr"/>
-      <c r="N28" t="inlineStr"/>
+      <c r="N28" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
       <c r="O28" t="inlineStr"/>
     </row>
     <row r="29"/>

</xml_diff>